<commit_message>
Deployed 255e4da with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Zeitlinie.xlsx
+++ b/Buch Bayrische Nächte/Zeitlinie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{074B868B-F1AC-409B-99A3-EFAF7C2913BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B437D2A-10C0-4FB1-AC11-5404F361E360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="90">
   <si>
     <t>Year</t>
   </si>
@@ -201,9 +201,6 @@
     <t>Aelxander goes to Munich to start studying at TUM at 16 years of age</t>
   </si>
   <si>
-    <t>Prologe</t>
-  </si>
-  <si>
     <t>Chaper 10</t>
   </si>
   <si>
@@ -233,16 +230,76 @@
     <t>Marina, Wilheml Freiherr, Philipp</t>
   </si>
   <si>
-    <t>Marina, Wilhelm, Philipp, Christoff, Gundel</t>
-  </si>
-  <si>
-    <t>Continuing Marina wakes up and remmebers the Coutns boat, searching in it for clues</t>
-  </si>
-  <si>
     <t>Marina, Gundel</t>
   </si>
   <si>
     <t>Josef, August, Ingenheim, Ashen-One, Lady of the Cult</t>
+  </si>
+  <si>
+    <t>Continuing Marina wakes up and remmebers the Counts boat, searching in it for clues</t>
+  </si>
+  <si>
+    <t>Friedrich, Marina, Alexander, Anna, Sabine, Helene Berthold, Nai, Sir Charles, etc.</t>
+  </si>
+  <si>
+    <t>Chapter 17</t>
+  </si>
+  <si>
+    <t>Chapter 14</t>
+  </si>
+  <si>
+    <t>Friedrich is talking with his demented mom about life</t>
+  </si>
+  <si>
+    <t>Friedrich, Walburga Pfeiffer</t>
+  </si>
+  <si>
+    <t>Marina, Wilhelm, Philipp, Christoff Bauer, Gundel Götz</t>
+  </si>
+  <si>
+    <t>Chapter 15</t>
+  </si>
+  <si>
+    <t>Chapter 13</t>
+  </si>
+  <si>
+    <t>Chapter 16</t>
+  </si>
+  <si>
+    <t>Chapter 18</t>
+  </si>
+  <si>
+    <t>Chapter 19</t>
+  </si>
+  <si>
+    <t>Chapter 21</t>
+  </si>
+  <si>
+    <t>Chapter 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meeting of the Wardens and </t>
+  </si>
+  <si>
+    <t>Murder on the Christmasmarket and ensuing chaos</t>
+  </si>
+  <si>
+    <t>Anna catches the killer while Alexander has visions through Maximilian</t>
+  </si>
+  <si>
+    <t>The Trio gets ist name and talks about their plans to make a decision</t>
+  </si>
+  <si>
+    <t>Anna gets trained by Sabine and learns about the Wardens</t>
+  </si>
+  <si>
+    <t>Josef and August learn more about the strange happenings around the Count von Tölz and run into Count von Ingenheim</t>
+  </si>
+  <si>
+    <t>Alexander wakes up from his visions</t>
+  </si>
+  <si>
+    <t>Alexander, Helene</t>
   </si>
 </sst>
 </file>
@@ -476,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.88671875" customWidth="1"/>
@@ -663,8 +720,11 @@
       <c r="C30">
         <v>25</v>
       </c>
+      <c r="D30" t="s">
+        <v>76</v>
+      </c>
       <c r="E30" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F30" t="s">
         <v>20</v>
@@ -709,7 +769,7 @@
         <v>22</v>
       </c>
       <c r="F36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -846,10 +906,10 @@
     </row>
     <row r="49" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="D49" t="s">
+        <v>57</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="F49" t="s">
         <v>50</v>
@@ -860,7 +920,7 @@
         <v>11</v>
       </c>
       <c r="D50" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>52</v>
@@ -871,24 +931,24 @@
     </row>
     <row r="51" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D51" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E51" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F51" t="s">
         <v>64</v>
-      </c>
-      <c r="F51" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="52" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D52" t="s">
+        <v>61</v>
+      </c>
+      <c r="E52" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E52" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="F52" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
     </row>
     <row r="53" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -896,19 +956,47 @@
         <v>12</v>
       </c>
       <c r="D53" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>68</v>
       </c>
       <c r="F53" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="54" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C54">
+        <v>13</v>
+      </c>
+      <c r="D54" t="s">
+        <v>78</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="55" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C55">
+        <v>16</v>
+      </c>
+      <c r="D55" t="s">
+        <v>71</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F55" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="56" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C56">
         <v>21</v>
       </c>
+      <c r="D56" t="s">
+        <v>75</v>
+      </c>
       <c r="E56" s="1" t="s">
         <v>54</v>
       </c>
@@ -918,18 +1006,79 @@
     </row>
     <row r="57" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C57">
+        <v>22</v>
+      </c>
+      <c r="D57" t="s">
+        <v>77</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="58" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C58">
+        <v>23</v>
+      </c>
+      <c r="D58" t="s">
+        <v>70</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="59" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C59">
         <v>24</v>
       </c>
-    </row>
-    <row r="58" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C58">
+      <c r="D59" t="s">
+        <v>79</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F59" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="60" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D60" t="s">
+        <v>81</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="61" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D61" t="s">
+        <v>80</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="62" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C62">
         <v>25</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="D62" t="s">
+        <v>3</v>
+      </c>
+      <c r="E62" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F58" t="s">
-        <v>70</v>
+      <c r="F62" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="63" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C63">
+        <v>27</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F63" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed a343614 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Zeitlinie.xlsx
+++ b/Buch Bayrische Nächte/Zeitlinie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B437D2A-10C0-4FB1-AC11-5404F361E360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301687EC-E6EF-41B7-BDEB-896471AB2670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="95">
   <si>
     <t>Year</t>
   </si>
@@ -82,28 +82,18 @@
 and only hers, capsized. Sir Charles was bheind that but no one knew. The Regatta was cancled in the following years.</t>
   </si>
   <si>
-    <t>Alexander and his brother Ludwig play on a hill. Ludwig dares himself to drive down the hill with top speed.
-Alexander cheers him up. Ludwig dies, falling of and hitting his head on a rock.</t>
-  </si>
-  <si>
     <t>June</t>
   </si>
   <si>
     <t>Friedrich, Maria sr.</t>
   </si>
   <si>
-    <t>Chapter 2</t>
-  </si>
-  <si>
     <t>Marina meets the Count Großberg to discuss the railcar project</t>
   </si>
   <si>
     <t>October</t>
   </si>
   <si>
-    <t>Chapter 3</t>
-  </si>
-  <si>
     <t>Alexander finalizes the plans for the railcar project</t>
   </si>
   <si>
@@ -119,9 +109,6 @@
     <t>December</t>
   </si>
   <si>
-    <t>Chapter 4</t>
-  </si>
-  <si>
     <t>Friedrich has an episode, that almost kills him</t>
   </si>
   <si>
@@ -134,16 +121,10 @@
     <t>Friedrich, Trautl, Elke, Maria jr.</t>
   </si>
   <si>
-    <t>Chapter 5</t>
-  </si>
-  <si>
     <t>The trio meets for the first time and ascents the mountain with the Count Großberg</t>
   </si>
   <si>
     <t>Friedrich, Marina, Alexander, Count Großberg</t>
-  </si>
-  <si>
-    <t>Chapter 6</t>
   </si>
   <si>
     <t>Marina studies the books of Großberg while the other ski. She finds out more about werewolves with Alexander. 
@@ -153,27 +134,18 @@
     <t>Friedrich, Marina, Alexander, Count Großberg, Eric</t>
   </si>
   <si>
-    <t>Chapter 7</t>
-  </si>
-  <si>
     <t>Breakfast and ski donw the slope. Friedrich hurts himself because of the other Count. A heavy storm begins. Count Großberg leaves them in the Storm and darts off.</t>
   </si>
   <si>
     <t>Friedrich, Marina, Alexander, Count Großberg, Eric, Count Ingenheim</t>
   </si>
   <si>
-    <t>Chapter 8</t>
-  </si>
-  <si>
     <t>Friedrich scouts the chalet grounds and finds the Werewolf. He hurts it badly but gets sliced himself. The others save him.</t>
   </si>
   <si>
     <t>Friedrich, Marina, Alexander, Werewolf, Eric</t>
   </si>
   <si>
-    <t>Chapter 9</t>
-  </si>
-  <si>
     <t>Marina and Alexander prepare for another Werewolf attack and have to fight against Eric. They beat him down and make themselves ready.</t>
   </si>
   <si>
@@ -183,9 +155,6 @@
     <t>Anna Siebert, Sabine, Karl</t>
   </si>
   <si>
-    <t>Chapter 1</t>
-  </si>
-  <si>
     <t>Josef Fuchsberger suspects foul play after the suspects releases</t>
   </si>
   <si>
@@ -196,12 +165,6 @@
   </si>
   <si>
     <t>Count von Ingenheim, Fuchsberger und August try to uncover the lies of the Trio but are caught in the Web of the Cult in the Karmeliterkirche next to the Christmas Market</t>
-  </si>
-  <si>
-    <t>Aelxander goes to Munich to start studying at TUM at 16 years of age</t>
-  </si>
-  <si>
-    <t>Chaper 10</t>
   </si>
   <si>
     <t>Sabine and Karl, Dianists of the Wardens, catch Anna Siebert in the villa of the Count Grossberg in Tölz</t>
@@ -211,12 +174,6 @@
 They talk about expectations of having a child.</t>
   </si>
   <si>
-    <t>Chapter 11</t>
-  </si>
-  <si>
-    <t>Chapter 12</t>
-  </si>
-  <si>
     <t>Marina arrives home with ehr huibsand Wilhelm, there she meets her son and attendance. She later has sex with her 
 husband to cope, bad dreams keeping her awake.</t>
   </si>
@@ -242,12 +199,6 @@
     <t>Friedrich, Marina, Alexander, Anna, Sabine, Helene Berthold, Nai, Sir Charles, etc.</t>
   </si>
   <si>
-    <t>Chapter 17</t>
-  </si>
-  <si>
-    <t>Chapter 14</t>
-  </si>
-  <si>
     <t>Friedrich is talking with his demented mom about life</t>
   </si>
   <si>
@@ -257,27 +208,6 @@
     <t>Marina, Wilhelm, Philipp, Christoff Bauer, Gundel Götz</t>
   </si>
   <si>
-    <t>Chapter 15</t>
-  </si>
-  <si>
-    <t>Chapter 13</t>
-  </si>
-  <si>
-    <t>Chapter 16</t>
-  </si>
-  <si>
-    <t>Chapter 18</t>
-  </si>
-  <si>
-    <t>Chapter 19</t>
-  </si>
-  <si>
-    <t>Chapter 21</t>
-  </si>
-  <si>
-    <t>Chapter 20</t>
-  </si>
-  <si>
     <t xml:space="preserve">Meeting of the Wardens and </t>
   </si>
   <si>
@@ -300,6 +230,90 @@
   </si>
   <si>
     <t>Alexander, Helene</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>Book1/13</t>
+  </si>
+  <si>
+    <t>Book1/1</t>
+  </si>
+  <si>
+    <t>Book1/2</t>
+  </si>
+  <si>
+    <t>Book1/3</t>
+  </si>
+  <si>
+    <t>Book1/4</t>
+  </si>
+  <si>
+    <t>Book1/5</t>
+  </si>
+  <si>
+    <t>Book1/6</t>
+  </si>
+  <si>
+    <t>Book1/7</t>
+  </si>
+  <si>
+    <t>Book1/8</t>
+  </si>
+  <si>
+    <t>Book1/9</t>
+  </si>
+  <si>
+    <t>Book1/10</t>
+  </si>
+  <si>
+    <t>Book1/17</t>
+  </si>
+  <si>
+    <t>Book1/11</t>
+  </si>
+  <si>
+    <t>Book1/12</t>
+  </si>
+  <si>
+    <t>Book1/18</t>
+  </si>
+  <si>
+    <t>Book1/14</t>
+  </si>
+  <si>
+    <t>Book1/15</t>
+  </si>
+  <si>
+    <t>Book1/16</t>
+  </si>
+  <si>
+    <t>Book1/19</t>
+  </si>
+  <si>
+    <t>Book1/20</t>
+  </si>
+  <si>
+    <t>Book1/21</t>
+  </si>
+  <si>
+    <t>Book1/</t>
+  </si>
+  <si>
+    <t>Alexander trying a 'science' experiment. Older schoolboys bully him for it and his brother Ludwig intervenes, sends Alexander away. He hides and hears his brother die on accident after a push, blacks it from his memories.</t>
+  </si>
+  <si>
+    <t>Alexander goes to Munich to start studying at TUM at 16 years of age</t>
+  </si>
+  <si>
+    <t>Friedrich and Maria talk again about their life together, he notices her frustration forthe first time.</t>
+  </si>
+  <si>
+    <t>Maria sr. Dies, killing herself with Friedrichs weaopn, as he walks away. He hears the shot from outside of their appartment</t>
+  </si>
+  <si>
+    <t>Alois Großbërge von Tolnzar becomes the Werewolf Fury</t>
   </si>
 </sst>
 </file>
@@ -533,12 +547,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.88671875" customWidth="1"/>
     <col min="4" max="4" width="10.44140625" customWidth="1"/>
-    <col min="5" max="5" width="105.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="109.5546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="70.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -562,6 +576,14 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1632</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
     <row r="4" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1850</v>
@@ -703,7 +725,7 @@
         <v>2</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>18</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -713,7 +735,7 @@
     </row>
     <row r="29" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -721,364 +743,401 @@
         <v>25</v>
       </c>
       <c r="D30" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="F30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>1871</v>
+        <v>1863</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>56</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A34">
-        <v>1882</v>
+      <c r="B34" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B35" t="s">
-        <v>14</v>
+      <c r="C35">
+        <v>6</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F35" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C36">
-        <v>10</v>
-      </c>
-      <c r="D36" t="s">
-        <v>51</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F36" t="s">
-        <v>65</v>
+      <c r="A36">
+        <v>1871</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C38">
-        <v>28</v>
-      </c>
-      <c r="D38" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F38" t="s">
-        <v>26</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C39">
-        <v>29</v>
-      </c>
-      <c r="D39" t="s">
-        <v>21</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F39" t="s">
-        <v>28</v>
+      <c r="A39">
+        <v>1882</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C41">
+        <v>10</v>
+      </c>
+      <c r="D41" t="s">
+        <v>69</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F41" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C43">
+        <v>28</v>
+      </c>
+      <c r="D43" t="s">
+        <v>70</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F43" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C44">
+        <v>29</v>
+      </c>
+      <c r="D44" t="s">
+        <v>70</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F44" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B45" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C46">
         <v>8</v>
       </c>
-      <c r="D41" t="s">
-        <v>24</v>
-      </c>
-      <c r="E41" s="1" t="s">
+      <c r="D46" t="s">
+        <v>71</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F46" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C47">
+        <v>9</v>
+      </c>
+      <c r="D47" t="s">
+        <v>71</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F47" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D48" t="s">
+        <v>72</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F48" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C42">
-        <v>9</v>
-      </c>
-      <c r="D42" t="s">
-        <v>24</v>
-      </c>
-      <c r="E42" s="1" t="s">
+    <row r="49" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D49" t="s">
+        <v>73</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F49" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D43" t="s">
-        <v>30</v>
-      </c>
-      <c r="E43" s="1" t="s">
+    <row r="50" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C50">
+        <v>10</v>
+      </c>
+      <c r="D50" t="s">
+        <v>74</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F50" t="s">
         <v>36</v>
       </c>
-      <c r="F43" t="s">
+    </row>
+    <row r="51" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D51" t="s">
+        <v>75</v>
+      </c>
+      <c r="E51" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D44" t="s">
-        <v>35</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F44" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C45">
-        <v>10</v>
-      </c>
-      <c r="D45" t="s">
+      <c r="F51" t="s">
         <v>38</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F45" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D46" t="s">
-        <v>41</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F46" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D47" t="s">
-        <v>44</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F47" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D48" t="s">
-        <v>47</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="49" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D49" t="s">
-        <v>57</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F49" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="50" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C50">
-        <v>11</v>
-      </c>
-      <c r="D50" t="s">
-        <v>70</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F50" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="51" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D51" t="s">
-        <v>60</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F51" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="52" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D52" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="F52" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="53" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C53">
-        <v>12</v>
-      </c>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="53" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D53" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F53" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="54" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C54">
-        <v>13</v>
-      </c>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="54" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="D54" t="s">
         <v>78</v>
       </c>
       <c r="E54" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F54" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="55" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C55">
+        <v>11</v>
+      </c>
+      <c r="D55" t="s">
+        <v>79</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F55" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="56" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D56" t="s">
+        <v>80</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F56" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="57" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D57" t="s">
+        <v>81</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F57" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="58" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C58">
+        <v>12</v>
+      </c>
+      <c r="D58" t="s">
+        <v>81</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F58" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C59">
+        <v>13</v>
+      </c>
+      <c r="D59" t="s">
+        <v>82</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="60" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C60">
+        <v>16</v>
+      </c>
+      <c r="D60" t="s">
+        <v>83</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F60" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="61" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C61">
+        <v>21</v>
+      </c>
+      <c r="D61" t="s">
+        <v>84</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F61" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="62" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C62">
+        <v>22</v>
+      </c>
+      <c r="D62" t="s">
+        <v>85</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="63" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C63">
+        <v>23</v>
+      </c>
+      <c r="D63" t="s">
+        <v>79</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="64" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C64">
+        <v>24</v>
+      </c>
+      <c r="D64" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="55" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C55">
-        <v>16</v>
-      </c>
-      <c r="D55" t="s">
-        <v>71</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F55" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="56" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C56">
-        <v>21</v>
-      </c>
-      <c r="D56" t="s">
-        <v>75</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F56" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="57" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C57">
-        <v>22</v>
-      </c>
-      <c r="D57" t="s">
-        <v>77</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="58" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C58">
-        <v>23</v>
-      </c>
-      <c r="D58" t="s">
-        <v>70</v>
-      </c>
-      <c r="E58" s="1" t="s">
+      <c r="E64" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F64" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="65" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D65" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="59" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C59">
-        <v>24</v>
-      </c>
-      <c r="D59" t="s">
-        <v>79</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F59" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="60" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D60" t="s">
-        <v>81</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="61" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D61" t="s">
-        <v>80</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="62" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C62">
+      <c r="E65" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D66" t="s">
+        <v>88</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="67" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C67">
         <v>25</v>
       </c>
-      <c r="D62" t="s">
-        <v>3</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F62" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="63" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C63">
+      <c r="D67" t="s">
+        <v>89</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F67" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="68" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C68">
         <v>27</v>
       </c>
-      <c r="E63" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F63" t="s">
+      <c r="D68" t="s">
         <v>89</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F68" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed d51faa1 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Zeitlinie.xlsx
+++ b/Buch Bayrische Nächte/Zeitlinie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEDF0791-F904-4ED4-9EB5-669DAC9107BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D6E2768-D94B-49C3-95F9-25142B5D96EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -195,9 +195,6 @@
     <t>Friedrich is talking with his demented mom about life</t>
   </si>
   <si>
-    <t>Friedrich, Walburga Pfeiffer</t>
-  </si>
-  <si>
     <t>Marina, Wilhelm, Philipp, Christoff Bauer, Gundel Götz</t>
   </si>
   <si>
@@ -320,6 +317,9 @@
   </si>
   <si>
     <t>Breakfast and ski down the slope. Friedrich hurts himself because of the other Count. A heavy storm begins. Count Großberg leaves them in the Storm and darts off.</t>
+  </si>
+  <si>
+    <t>Friedrich, Waltraut Pfeiffer</t>
   </si>
 </sst>
 </file>
@@ -587,7 +587,7 @@
         <v>1632</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -731,7 +731,7 @@
         <v>2</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -749,7 +749,7 @@
         <v>25</v>
       </c>
       <c r="D30" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>46</v>
@@ -765,7 +765,7 @@
     </row>
     <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -773,7 +773,7 @@
         <v>2</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -786,7 +786,7 @@
         <v>6</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F35" t="s">
         <v>19</v>
@@ -807,7 +807,7 @@
         <v>3</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -825,7 +825,7 @@
         <v>10</v>
       </c>
       <c r="D41" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>20</v>
@@ -844,7 +844,7 @@
         <v>28</v>
       </c>
       <c r="D43" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>22</v>
@@ -858,7 +858,7 @@
         <v>29</v>
       </c>
       <c r="D44" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>24</v>
@@ -877,7 +877,7 @@
         <v>8</v>
       </c>
       <c r="D46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>27</v>
@@ -891,7 +891,7 @@
         <v>9</v>
       </c>
       <c r="D47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>29</v>
@@ -902,7 +902,7 @@
     </row>
     <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="D48" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>31</v>
@@ -913,7 +913,7 @@
     </row>
     <row r="49" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D49" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>33</v>
@@ -927,10 +927,10 @@
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F50" t="s">
         <v>35</v>
@@ -938,7 +938,7 @@
     </row>
     <row r="51" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="D51" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>36</v>
@@ -949,7 +949,7 @@
     </row>
     <row r="52" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D52" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>38</v>
@@ -960,7 +960,7 @@
     </row>
     <row r="53" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D53" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>39</v>
@@ -968,7 +968,7 @@
     </row>
     <row r="54" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="D54" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>45</v>
@@ -982,7 +982,7 @@
         <v>11</v>
       </c>
       <c r="D55" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>41</v>
@@ -993,7 +993,7 @@
     </row>
     <row r="56" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D56" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>47</v>
@@ -1004,13 +1004,13 @@
     </row>
     <row r="57" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D57" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F57" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="58" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1018,7 +1018,7 @@
         <v>12</v>
       </c>
       <c r="D58" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>52</v>
@@ -1032,10 +1032,10 @@
         <v>13</v>
       </c>
       <c r="D59" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="60" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1043,13 +1043,13 @@
         <v>16</v>
       </c>
       <c r="D60" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>54</v>
       </c>
       <c r="F60" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
     </row>
     <row r="61" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -1057,7 +1057,7 @@
         <v>21</v>
       </c>
       <c r="D61" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>43</v>
@@ -1071,10 +1071,10 @@
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="63" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -1082,18 +1082,18 @@
         <v>23</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="64" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="D64" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E64" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="65" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -1101,10 +1101,10 @@
         <v>24</v>
       </c>
       <c r="D65" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F65" t="s">
         <v>53</v>
@@ -1112,18 +1112,18 @@
     </row>
     <row r="66" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="D66" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="67" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="D67" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="68" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -1131,7 +1131,7 @@
         <v>25</v>
       </c>
       <c r="D68" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>44</v>
@@ -1145,13 +1145,13 @@
         <v>27</v>
       </c>
       <c r="D69" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E69" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F69" t="s">
         <v>63</v>
-      </c>
-      <c r="F69" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed e518e35 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Zeitlinie.xlsx
+++ b/Buch Bayrische Nächte/Zeitlinie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D6E2768-D94B-49C3-95F9-25142B5D96EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2D3369-40BE-46C7-A35D-2C6E2A871411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="100">
   <si>
     <t>Year</t>
   </si>
@@ -320,6 +320,15 @@
   </si>
   <si>
     <t>Friedrich, Waltraut Pfeiffer</t>
+  </si>
+  <si>
+    <t>Michael wants to kill himself but falters. Ends up saving Maximilian from Temprests  and vows to keep going.</t>
+  </si>
+  <si>
+    <t>Michael, Maximilian</t>
+  </si>
+  <si>
+    <t>Michaels wife Bärbel dies of stomach cancer and he loses hope, vanishes from sight for half a year. His brewery is continued running by his staff and brewmaster.</t>
   </si>
 </sst>
 </file>
@@ -553,7 +562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.88671875" customWidth="1"/>
@@ -812,345 +821,384 @@
     </row>
     <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>1882</v>
+        <v>1880</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C41">
+        <v>8</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>1881</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B43" t="s">
         <v>10</v>
-      </c>
-      <c r="D41" t="s">
-        <v>66</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F41" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B42" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C43">
-        <v>28</v>
-      </c>
-      <c r="D43" t="s">
-        <v>67</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F43" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C44">
-        <v>29</v>
-      </c>
-      <c r="D44" t="s">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>24</v>
+        <v>97</v>
       </c>
       <c r="F44" t="s">
-        <v>25</v>
+        <v>98</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B45" t="s">
-        <v>26</v>
+      <c r="A45">
+        <v>1882</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C46">
-        <v>8</v>
-      </c>
-      <c r="D46" t="s">
-        <v>68</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F46" t="s">
-        <v>28</v>
+      <c r="B46" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C47">
+        <v>10</v>
+      </c>
+      <c r="D47" t="s">
+        <v>66</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F47" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B48" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C49">
+        <v>28</v>
+      </c>
+      <c r="D49" t="s">
+        <v>67</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F49" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C50">
+        <v>29</v>
+      </c>
+      <c r="D50" t="s">
+        <v>67</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F50" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B51" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C52">
+        <v>8</v>
+      </c>
+      <c r="D52" t="s">
+        <v>68</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F52" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C53">
         <v>9</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D53" t="s">
         <v>68</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="E53" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F53" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D48" t="s">
+    <row r="54" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D54" t="s">
         <v>69</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="E54" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F54" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="49" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D49" t="s">
+    <row r="55" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D55" t="s">
         <v>70</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E55" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F55" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="50" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C50">
+    <row r="56" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C56">
         <v>10</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D56" t="s">
         <v>71</v>
       </c>
-      <c r="E50" s="1" t="s">
+      <c r="E56" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="F50" t="s">
+      <c r="F56" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D51" t="s">
+    <row r="57" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D57" t="s">
         <v>72</v>
       </c>
-      <c r="E51" s="1" t="s">
+      <c r="E57" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F57" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="52" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D52" t="s">
+    <row r="58" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D58" t="s">
         <v>73</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E58" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F58" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="53" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D53" t="s">
+    <row r="59" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D59" t="s">
         <v>74</v>
       </c>
-      <c r="E53" s="1" t="s">
+      <c r="E59" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="54" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D54" t="s">
+    <row r="60" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D60" t="s">
         <v>75</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="E60" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F54" t="s">
+      <c r="F60" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="55" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C55">
+    <row r="61" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C61">
         <v>11</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D61" t="s">
         <v>76</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="E61" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F61" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D56" t="s">
+    <row r="62" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D62" t="s">
         <v>77</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="E62" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F62" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="57" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D57" t="s">
+    <row r="63" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D63" t="s">
         <v>78</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="E63" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="F57" t="s">
+      <c r="F63" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C58">
+    <row r="64" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C64">
         <v>12</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D64" t="s">
         <v>78</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="E64" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F58" t="s">
+      <c r="F64" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="59" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C59">
+    <row r="65" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C65">
         <v>13</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D65" t="s">
         <v>79</v>
       </c>
-      <c r="E59" s="1" t="s">
+      <c r="E65" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="60" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C60">
+    <row r="66" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C66">
         <v>16</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D66" t="s">
         <v>80</v>
       </c>
-      <c r="E60" s="1" t="s">
+      <c r="E66" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F60" t="s">
+      <c r="F66" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="61" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C61">
+    <row r="67" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C67">
         <v>21</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D67" t="s">
         <v>81</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="E67" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F67" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C62">
+    <row r="68" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C68">
         <v>22</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D68" t="s">
         <v>82</v>
       </c>
-      <c r="E62" s="1" t="s">
+      <c r="E68" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C63">
+    <row r="69" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C69">
         <v>23</v>
       </c>
-      <c r="D63" s="1" t="s">
+      <c r="D69" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E63" s="1" t="s">
+      <c r="E69" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="64" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D64" s="1" t="s">
+    <row r="70" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D70" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="E70" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="65" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C65">
+    <row r="71" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C71">
         <v>24</v>
       </c>
-      <c r="D65" t="s">
+      <c r="D71" t="s">
         <v>83</v>
       </c>
-      <c r="E65" s="1" t="s">
+      <c r="E71" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F65" t="s">
+      <c r="F71" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="66" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D66" t="s">
+    <row r="72" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D72" t="s">
         <v>84</v>
       </c>
-      <c r="E66" s="1" t="s">
+      <c r="E72" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="67" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="D67" t="s">
+    <row r="73" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D73" t="s">
         <v>85</v>
       </c>
-      <c r="E67" s="1" t="s">
+      <c r="E73" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="68" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C68">
+    <row r="74" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C74">
         <v>25</v>
       </c>
-      <c r="D68" t="s">
+      <c r="D74" t="s">
         <v>86</v>
       </c>
-      <c r="E68" s="1" t="s">
+      <c r="E74" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F68" t="s">
+      <c r="F74" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="69" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C69">
+    <row r="75" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C75">
         <v>27</v>
       </c>
-      <c r="D69" t="s">
+      <c r="D75" t="s">
         <v>86</v>
       </c>
-      <c r="E69" s="1" t="s">
+      <c r="E75" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F69" t="s">
+      <c r="F75" t="s">
         <v>63</v>
       </c>
     </row>

</xml_diff>